<commit_message>
En cas de rencontre, implémenter les fonctions Commercer,Poursuivre,PavillonNoir et Canonner dans voyage à partir de la méthode executer actions ligne 287
Bug ajout trait PNJ résolu
</commit_message>
<xml_diff>
--- a/files/data/Traits.xlsx
+++ b/files/data/Traits.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/054f950197fbca64/Documents/Jeu/PavillonNoirLogiciel/LogicielPNGaming/files/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="5" documentId="13_ncr:1_{B2AD58D5-8BDD-4C77-9363-2DBF5497C755}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E9881579-1E60-4DF7-9EE8-C42CE7D36A20}"/>
+  <xr:revisionPtr revIDLastSave="11" documentId="13_ncr:1_{B2AD58D5-8BDD-4C77-9363-2DBF5497C755}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0B2B29DF-E1AA-43E2-81D9-104C1D2FA662}"/>
   <bookViews>
-    <workbookView xWindow="588" yWindow="13548" windowWidth="21600" windowHeight="11292" xr2:uid="{18E8458F-5FC7-40D3-B3A0-FCFA88649893}"/>
+    <workbookView xWindow="-108" yWindow="12852" windowWidth="23256" windowHeight="12456" xr2:uid="{18E8458F-5FC7-40D3-B3A0-FCFA88649893}"/>
   </bookViews>
   <sheets>
     <sheet name="Feuil1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="77" uniqueCount="72">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="81" uniqueCount="76">
   <si>
     <t>Col</t>
   </si>
@@ -241,6 +241,18 @@
   </si>
   <si>
     <t>InterprèteNeerlandais</t>
+  </si>
+  <si>
+    <t>Navigation</t>
+  </si>
+  <si>
+    <t>Navigateur</t>
+  </si>
+  <si>
+    <t>Hydrographie</t>
+  </si>
+  <si>
+    <t>Hydrographe</t>
   </si>
 </sst>
 </file>
@@ -612,7 +624,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0530DE92-7D37-4C1A-BDF3-4A4B6A10D1E0}">
-  <dimension ref="A1:C38"/>
+  <dimension ref="A1:C40"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
@@ -1033,6 +1045,28 @@
         <v>67</v>
       </c>
     </row>
+    <row r="39" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A39" t="s">
+        <v>72</v>
+      </c>
+      <c r="B39">
+        <v>2</v>
+      </c>
+      <c r="C39" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="40" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A40" t="s">
+        <v>74</v>
+      </c>
+      <c r="B40">
+        <v>2</v>
+      </c>
+      <c r="C40" t="s">
+        <v>75</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>